<commit_message>
Record Mesh 2 baseline mesh-independence data (workbook + log)
</commit_message>
<xml_diff>
--- a/thesis/mesh-validation/Baseline_Smooth_Mesh_Independence_Workbook.xlsx
+++ b/thesis/mesh-validation/Baseline_Smooth_Mesh_Independence_Workbook.xlsx
@@ -1431,8 +1431,6 @@
           <t>Intensity and Hydraulic Diameter</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1448,7 +1446,6 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1481,7 +1478,6 @@
           <t>≈ 99,800</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Matches enhanced-geometry Coarse level's own logged Re≈99,600</t>
@@ -1955,13 +1951,21 @@
       <c r="B5" s="6" t="n">
         <v>3.85</v>
       </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
+      <c r="C5" s="6" t="n">
+        <v>1762070</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>650727</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.84496</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.15504</v>
+      </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Recorded 2026-08-19, same convention as Mesh 1 (Re=100,000, Tin=300K, uniform q"=1000 W/m2)</t>
         </is>
       </c>
     </row>
@@ -2171,6 +2175,45 @@
           <t>Mesh 2</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>452.23211</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.3359388</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-4.3359386</v>
+      </c>
+      <c r="E5" t="n">
+        <v>640.89111</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>300</v>
+      </c>
+      <c r="H5" t="n">
+        <v>300.05315</v>
+      </c>
+      <c r="I5" t="n">
+        <v>300.86581</v>
+      </c>
+      <c r="J5" t="n">
+        <v>6.0110973</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.27043937</v>
+      </c>
+      <c r="M5" t="n">
+        <v>2.1768591</v>
+      </c>
+      <c r="N5" t="n">
+        <v>5e-06</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">

</xml_diff>

<commit_message>
Record Mesh 3 baseline mesh-independence data; not yet converged, proceed to Mesh 4
</commit_message>
<xml_diff>
--- a/thesis/mesh-validation/Baseline_Smooth_Mesh_Independence_Workbook.xlsx
+++ b/thesis/mesh-validation/Baseline_Smooth_Mesh_Independence_Workbook.xlsx
@@ -1978,13 +1978,21 @@
       <c r="B6" s="6" t="n">
         <v>2.96</v>
       </c>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
+      <c r="C6" s="6" t="n">
+        <v>3093142</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>1117290</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.84995</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0.15005</v>
+      </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Recorded 2026-08-19, same convention as Mesh 1/2</t>
         </is>
       </c>
     </row>
@@ -2221,6 +2229,45 @@
           <t>Mesh 3</t>
         </is>
       </c>
+      <c r="B6" t="n">
+        <v>452.29636</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.3399049</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-4.3399046</v>
+      </c>
+      <c r="E6" t="n">
+        <v>598.08387</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>300</v>
+      </c>
+      <c r="H6" t="n">
+        <v>300.05311</v>
+      </c>
+      <c r="I6" t="n">
+        <v>300.85761</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5.9357157</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.27342043</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1.4947357</v>
+      </c>
+      <c r="N6" t="n">
+        <v>7e-06</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>

<commit_message>
Record Mesh 4 baseline data; ΔP still 2.57%, extend to Mesh 5
</commit_message>
<xml_diff>
--- a/thesis/mesh-validation/Baseline_Smooth_Mesh_Independence_Workbook.xlsx
+++ b/thesis/mesh-validation/Baseline_Smooth_Mesh_Independence_Workbook.xlsx
@@ -2005,14 +2005,32 @@
       <c r="B7" s="6" t="n">
         <v>2.28</v>
       </c>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
+      <c r="C7" s="6" t="n">
+        <v>5825667</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>1986806</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.79995</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.20005</v>
+      </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Pending, if needed</t>
-        </is>
+          <t>Recorded 2026-08-19, same convention as Mesh 1/2/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Mesh 5 (extra level, ΔP not yet converged at Mesh 4)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1.75</v>
       </c>
     </row>
     <row r="9">
@@ -2033,7 +2051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2273,6 +2291,52 @@
       <c r="A7" t="inlineStr">
         <is>
           <t>Mesh 4</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>452.33431</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.3422859</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-4.3422856</v>
+      </c>
+      <c r="E7" t="n">
+        <v>583.1092599999999</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>300</v>
+      </c>
+      <c r="H7" t="n">
+        <v>300.05309</v>
+      </c>
+      <c r="I7" t="n">
+        <v>300.86379</v>
+      </c>
+      <c r="J7" t="n">
+        <v>6.0018683</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.27537764</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1.5131235</v>
+      </c>
+      <c r="N7" t="n">
+        <v>7e-06</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Mesh 5</t>
         </is>
       </c>
     </row>
@@ -2669,6 +2733,53 @@
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mesh 5</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>IF('Fluent Raw Results'!C8="","",'Fluent Raw Results'!C8/($B$7*$B$5))</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>IF('Fluent Raw Results'!C8="","",$B$7*B17*$B$4/$B$8)</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>IF('Fluent Raw Results'!G8="","",('Fluent Raw Results'!G8+'Fluent Raw Results'!H8)/2)</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>IF(OR('Fluent Raw Results'!I8="",D17=""),"",'Fluent Raw Results'!K8/('Fluent Raw Results'!I8-D17))</f>
+        <v/>
+      </c>
+      <c r="F17">
+        <f>IF(E17="","",E17*$B$4/$B$9)</f>
+        <v/>
+      </c>
+      <c r="G17">
+        <f>IF(OR('Fluent Raw Results'!J8="",B17=""),"",2*'Fluent Raw Results'!J8/($B$7*B17^2))</f>
+        <v/>
+      </c>
+      <c r="H17">
+        <f>IF(G17="","",4*G17*($B$6/$B$4)*($B$7*B17^2/2))</f>
+        <v/>
+      </c>
+      <c r="I17">
+        <f>IF('Fluent Raw Results'!E8="","",'Fluent Raw Results'!E8-'Fluent Raw Results'!F8)</f>
+        <v/>
+      </c>
+      <c r="J17">
+        <f>IF(OR(H17="",I17=""),"",ABS(H17-I17)/I17*100)</f>
+        <v/>
+      </c>
+      <c r="K17">
+        <f>IF('Fluent Raw Results'!N8="","",'Fluent Raw Results'!N8)</f>
+        <v/>
+      </c>
+    </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
@@ -2690,7 +2801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2861,6 +2972,41 @@
       </c>
       <c r="H8">
         <f>IF(OR(D8="",G8=""),"pending",IF(AND(D8&lt;2,G8&lt;2),"PASS","FAIL — needs finer mesh"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Mesh 4 -&gt; Mesh 5</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>'Computed Results'!F16</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>'Computed Results'!F17</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>IF(OR(B9="",C9=""),"",ABS(C9-B9)/C9*100)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>'Computed Results'!I16</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>'Computed Results'!I17</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>IF(OR(E9="",F9=""),"",ABS(F9-E9)/F9*100)</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>IF(OR(D9="",G9=""),"pending",IF(AND(D9&lt;2,G9&lt;2),"PASS","FAIL — needs finer mesh"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark Mesh 4 as provisionally adopted; flag old Mesh-1 production run as superseded
</commit_message>
<xml_diff>
--- a/thesis/mesh-validation/Baseline_Smooth_Mesh_Independence_Workbook.xlsx
+++ b/thesis/mesh-validation/Baseline_Smooth_Mesh_Independence_Workbook.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +56,10 @@
     <font>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
     </font>
   </fonts>
   <fills count="3">
@@ -97,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +119,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -482,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -645,13 +652,28 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Status (2026-08-19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Mesh 4 PROVISIONALLY ADOPTED. Mesh 3-&gt;4: Nu PASS (0.75%), dP FAIL (2.57%, just above 2%). Mesh 5 in progress to confirm. Production work (Baseline run + Run 2+) proceeding on Mesh 4 in the meantime; will revisit only if Mesh 5 shows a material further change.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B11:F11"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B9:F9"/>
@@ -3046,9 +3068,9 @@
       </c>
     </row>
     <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Completed 2026-08-19 on the same Mesh 1 geometry/mesh as the mesh-independence test above, but with REAL production boundary conditions — NOT part of the mesh-independence comparison. Saved here for reuse once mesh independence is formally established and the final adopted mesh level is known.</t>
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>SUPERSEDED: this data was run on Mesh 1 geometry, before mesh independence was checked. Now that Mesh 4 is (provisionally) adopted, this run must be redone on Mesh 4 before use in the 27-run master workbook. Kept below for reference only.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Baseline mesh independence achieved: Mesh 4 adopted, confirmed by Mesh 5
</commit_message>
<xml_diff>
--- a/thesis/mesh-validation/Baseline_Smooth_Mesh_Independence_Workbook.xlsx
+++ b/thesis/mesh-validation/Baseline_Smooth_Mesh_Independence_Workbook.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +60,10 @@
     <font>
       <b val="1"/>
       <color rgb="00C00000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
     </font>
   </fonts>
   <fills count="3">
@@ -101,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -124,6 +128,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -666,8 +671,22 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>FINAL VERDICT (2026-08-19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Mesh independence ACHIEVED. Mesh 4 -&gt; Mesh 5: Nu 1.57% PASS, dP 0.46% PASS. Mesh 4 (2.28mm, 5,825,667 elements) is the adopted baseline mesh (Mesh 5 only confirmed it). Next: re-run real production Baseline conditions on Mesh 4, log into the 27-run master workbook.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B6:F6"/>
@@ -678,6 +697,7 @@
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B13:F13"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2048,11 +2068,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mesh 5 (extra level, ΔP not yet converged at Mesh 4)</t>
+          <t>Mesh 5</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>1.75</v>
+      </c>
+      <c r="C8" t="n">
+        <v>10148909</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3414651</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.79664</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.20336</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Recorded 2026-08-19, same convention as Mesh 1-4</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -2361,6 +2398,45 @@
           <t>Mesh 5</t>
         </is>
       </c>
+      <c r="B8" t="n">
+        <v>452.3567</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.3436847</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-4.3436845</v>
+      </c>
+      <c r="E8" t="n">
+        <v>580.41596</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>300</v>
+      </c>
+      <c r="H8" t="n">
+        <v>300.05308</v>
+      </c>
+      <c r="I8" t="n">
+        <v>300.85067</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6.1272085</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.2786611</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1.6291049</v>
+      </c>
+      <c r="N8" t="n">
+        <v>5e-06</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>